<commit_message>
October Dispatch finalized; transit research numbers and To and Fro town stops refresh
</commit_message>
<xml_diff>
--- a/research/files/bc_transit_routes.xlsx
+++ b/research/files/bc_transit_routes.xlsx
@@ -11433,7 +11433,7 @@
         </is>
       </c>
       <c r="G192" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H192" t="inlineStr">
         <is>
@@ -12542,11 +12542,11 @@
         </is>
       </c>
       <c r="G211" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>Vanderhoof</t>
+          <t>Burns Lake</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -12598,7 +12598,7 @@
         </is>
       </c>
       <c r="G212" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -12715,7 +12715,7 @@
         </is>
       </c>
       <c r="G214" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H214" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         </is>
       </c>
       <c r="G231" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H231" t="inlineStr">
         <is>
@@ -13763,7 +13763,7 @@
         </is>
       </c>
       <c r="G232" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H232" t="inlineStr">
         <is>
@@ -13824,7 +13824,7 @@
         </is>
       </c>
       <c r="G233" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -13885,7 +13885,7 @@
         </is>
       </c>
       <c r="G234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
@@ -15050,7 +15050,7 @@
         </is>
       </c>
       <c r="G254" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -15172,7 +15172,7 @@
         </is>
       </c>
       <c r="G256" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -15181,7 +15181,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Central Saanich</t>
+          <t>Brentwood Bay (Vancouver Island)</t>
         </is>
       </c>
       <c r="J256" t="b">
@@ -15289,7 +15289,7 @@
         </is>
       </c>
       <c r="G258" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>

</xml_diff>